<commit_message>
Refactor: Standardize CRISP-DM headers, update PCA analysis, and sync .ipynb with .py
</commit_message>
<xml_diff>
--- a/clustering/Hasil_Profiling_Centroid.xlsx
+++ b/clustering/Hasil_Profiling_Centroid.xlsx
@@ -7,7 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semua_Parameter" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabel_1_Perolehan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabel_2_Partisipasi" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -731,4 +733,396 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>cluster_label</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>jumlah_kecamatan</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>persen_pilpres</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>persen_pileg_ri</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>persen_pileg_prov</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>persen_pileg_kokab</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>persen_pilgub</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>persen_pilwalbup</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="n">
+        <v>202</v>
+      </c>
+      <c r="C2" t="n">
+        <v>54.141</v>
+      </c>
+      <c r="D2" t="n">
+        <v>13.848</v>
+      </c>
+      <c r="E2" t="n">
+        <v>14.857</v>
+      </c>
+      <c r="F2" t="n">
+        <v>12.793</v>
+      </c>
+      <c r="G2" t="n">
+        <v>57.497</v>
+      </c>
+      <c r="H2" t="n">
+        <v>44.232</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="n">
+        <v>143</v>
+      </c>
+      <c r="C3" t="n">
+        <v>64.91200000000001</v>
+      </c>
+      <c r="D3" t="n">
+        <v>13.402</v>
+      </c>
+      <c r="E3" t="n">
+        <v>14.889</v>
+      </c>
+      <c r="F3" t="n">
+        <v>11.358</v>
+      </c>
+      <c r="G3" t="n">
+        <v>68.953</v>
+      </c>
+      <c r="H3" t="n">
+        <v>51.681</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="n">
+        <v>157</v>
+      </c>
+      <c r="C4" t="n">
+        <v>59.923</v>
+      </c>
+      <c r="D4" t="n">
+        <v>16.724</v>
+      </c>
+      <c r="E4" t="n">
+        <v>16.73</v>
+      </c>
+      <c r="F4" t="n">
+        <v>15.846</v>
+      </c>
+      <c r="G4" t="n">
+        <v>59.414</v>
+      </c>
+      <c r="H4" t="n">
+        <v>35.179</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="n">
+        <v>27</v>
+      </c>
+      <c r="C5" t="n">
+        <v>49.692</v>
+      </c>
+      <c r="D5" t="n">
+        <v>14.33</v>
+      </c>
+      <c r="E5" t="n">
+        <v>11.845</v>
+      </c>
+      <c r="F5" t="n">
+        <v>11.503</v>
+      </c>
+      <c r="G5" t="n">
+        <v>56.904</v>
+      </c>
+      <c r="H5" t="n">
+        <v>89.899</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="n">
+        <v>98</v>
+      </c>
+      <c r="C6" t="n">
+        <v>64.717</v>
+      </c>
+      <c r="D6" t="n">
+        <v>25.246</v>
+      </c>
+      <c r="E6" t="n">
+        <v>25.469</v>
+      </c>
+      <c r="F6" t="n">
+        <v>21.366</v>
+      </c>
+      <c r="G6" t="n">
+        <v>68.768</v>
+      </c>
+      <c r="H6" t="n">
+        <v>51.819</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>cluster_label</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>jumlah_kecamatan</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>persen_part_pilpres</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>persen_part_pileg_ri</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>persen_part_pileg_prov</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>persen_part_pileg_kokab</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>persen_part_pilgub</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>persen_part_pilwalbup</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>persen_baseline_pilwalbup</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="n">
+        <v>202</v>
+      </c>
+      <c r="C2" t="n">
+        <v>82.544</v>
+      </c>
+      <c r="D2" t="n">
+        <v>82.027</v>
+      </c>
+      <c r="E2" t="n">
+        <v>81.973</v>
+      </c>
+      <c r="F2" t="n">
+        <v>81.925</v>
+      </c>
+      <c r="G2" t="n">
+        <v>64.39700000000001</v>
+      </c>
+      <c r="H2" t="n">
+        <v>63.853</v>
+      </c>
+      <c r="I2" t="n">
+        <v>36.906</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="n">
+        <v>143</v>
+      </c>
+      <c r="C3" t="n">
+        <v>85.38</v>
+      </c>
+      <c r="D3" t="n">
+        <v>85.202</v>
+      </c>
+      <c r="E3" t="n">
+        <v>85.315</v>
+      </c>
+      <c r="F3" t="n">
+        <v>85.23099999999999</v>
+      </c>
+      <c r="G3" t="n">
+        <v>74.405</v>
+      </c>
+      <c r="H3" t="n">
+        <v>74.376</v>
+      </c>
+      <c r="I3" t="n">
+        <v>39.499</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="n">
+        <v>157</v>
+      </c>
+      <c r="C4" t="n">
+        <v>75.182</v>
+      </c>
+      <c r="D4" t="n">
+        <v>75.06699999999999</v>
+      </c>
+      <c r="E4" t="n">
+        <v>74.965</v>
+      </c>
+      <c r="F4" t="n">
+        <v>74.947</v>
+      </c>
+      <c r="G4" t="n">
+        <v>60.196</v>
+      </c>
+      <c r="H4" t="n">
+        <v>59.707</v>
+      </c>
+      <c r="I4" t="n">
+        <v>36.412</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="n">
+        <v>27</v>
+      </c>
+      <c r="C5" t="n">
+        <v>80.685</v>
+      </c>
+      <c r="D5" t="n">
+        <v>80.50700000000001</v>
+      </c>
+      <c r="E5" t="n">
+        <v>81.005</v>
+      </c>
+      <c r="F5" t="n">
+        <v>80.10899999999999</v>
+      </c>
+      <c r="G5" t="n">
+        <v>71.04600000000001</v>
+      </c>
+      <c r="H5" t="n">
+        <v>70.94</v>
+      </c>
+      <c r="I5" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="n">
+        <v>98</v>
+      </c>
+      <c r="C6" t="n">
+        <v>84.73999999999999</v>
+      </c>
+      <c r="D6" t="n">
+        <v>84.491</v>
+      </c>
+      <c r="E6" t="n">
+        <v>84.47</v>
+      </c>
+      <c r="F6" t="n">
+        <v>84.40600000000001</v>
+      </c>
+      <c r="G6" t="n">
+        <v>70.89100000000001</v>
+      </c>
+      <c r="H6" t="n">
+        <v>70.551</v>
+      </c>
+      <c r="I6" t="n">
+        <v>38.044</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>